<commit_message>
conditioned based constraints added
</commit_message>
<xml_diff>
--- a/outputs/final_open_shop/results/pyomo_same_case_results.xlsx
+++ b/outputs/final_open_shop/results/pyomo_same_case_results.xlsx
@@ -481,10 +481,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="G2" t="n">
-        <v>0.225</v>
+        <v>0.229</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>

</xml_diff>